<commit_message>
Add 'no child' option and new product suggestion
</commit_message>
<xml_diff>
--- a/Quizbot/data/INTRO.xlsx
+++ b/Quizbot/data/INTRO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\++My Codes\Web Develop\Telegam_Bale Bot\Keramat_Quizbot2\Quizbot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3201E86-7601-4A63-B636-17E273D21A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F0FF76B-BAA9-430B-84F8-50194913294A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="29">
   <si>
     <t>q_key</t>
   </si>
@@ -103,13 +103,22 @@
   </si>
   <si>
     <t>وضعیت تاهل خودتونو انتخاب کنین💍</t>
+  </si>
+  <si>
+    <t>no_child</t>
+  </si>
+  <si>
+    <t>بدون فرزند</t>
+  </si>
+  <si>
+    <t>none</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -117,13 +126,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0F1115"/>
+      <name val="Inter"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0F1115"/>
+      <name val="Inter"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -138,8 +165,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -442,7 +475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="7" width="40" customWidth="1"/>
@@ -599,7 +632,26 @@
         <v>21</v>
       </c>
     </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="1"/>
+      <c r="F9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Change Intro option text
</commit_message>
<xml_diff>
--- a/Quizbot/data/INTRO.xlsx
+++ b/Quizbot/data/INTRO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\++My Codes\Web Develop\Telegam_Bale Bot\Keramat_Quizbot2\Quizbot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F0FF76B-BAA9-430B-84F8-50194913294A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11712F02-58EF-4CF4-BD48-85EAF26E6B6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,18 +54,12 @@
     <t>single</t>
   </si>
   <si>
-    <t>مامان هستم</t>
-  </si>
-  <si>
     <t>mother</t>
   </si>
   <si>
     <t>female</t>
   </si>
   <si>
-    <t>بابا هستم</t>
-  </si>
-  <si>
     <t>father</t>
   </si>
   <si>
@@ -112,6 +106,12 @@
   </si>
   <si>
     <t>none</t>
+  </si>
+  <si>
+    <t>خانم متاهل هستم</t>
+  </si>
+  <si>
+    <t>آقای متاهل هستم</t>
   </si>
 </sst>
 </file>
@@ -509,16 +509,16 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -526,16 +526,16 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
         <v>8</v>
@@ -546,19 +546,19 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>10</v>
       </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
       <c r="G4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -566,88 +566,88 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
         <v>12</v>
       </c>
-      <c r="D5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" t="s">
-        <v>14</v>
-      </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
         <v>15</v>
       </c>
-      <c r="B6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" t="s">
-        <v>17</v>
-      </c>
       <c r="G6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>